<commit_message>
docs(tm): default the protocol to all roles on, no manual switches (v3.5)
</commit_message>
<xml_diff>
--- a/协作/模板/18-专项审查报告.xlsx
+++ b/协作/模板/18-专项审查报告.xlsx
@@ -2103,11 +2103,11 @@
     <dataValidation sqref="D2:D121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="只能选择下拉里的值" type="list">
       <formula1>"PASS,FAIL"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="只能选择下拉里的值" type="list">
-      <formula1>"安全,性能,供应链"</formula1>
-    </dataValidation>
     <dataValidation sqref="E2:E121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="取值不合法" error="只能选择下拉里的值" type="list">
       <formula1>"致命,严重,一般"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"安全,性能,供应链,兼容性,可运维性"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2136,6 +2136,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2208,6 +2209,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -2311,6 +2313,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
@@ -2582,6 +2585,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
@@ -2609,7 +2613,7 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>安全 / 性能 / 供应链</t>
+          <t>安全 / 性能 / 供应链 / 兼容性 / 可运维性</t>
         </is>
       </c>
     </row>

</xml_diff>